<commit_message>
fix(templates): actualizar plantillas oficiales de OT Suelo y Agregado y Recepcion Suelo y Agregado
</commit_message>
<xml_diff>
--- a/app/templates/OT/OT-SU-Y-AG/OT-0000-Geofal.xlsx
+++ b/app/templates/OT/OT-SU-Y-AG/OT-0000-Geofal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Equipo\Desktop\miguel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\OT\OT-SU-Y-AG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF42323B-E471-4BE8-A767-46DF73995611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D30F3E-C883-4009-89AB-A80F22AE44C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7CAA3784-AC6A-4491-9DAE-0EC89CC1DDD5}"/>
   </bookViews>
@@ -94,9 +94,6 @@
     <t>CODIGO ENSAYO</t>
   </si>
   <si>
-    <t>OT DESIGADA A:                                           (Nnombre del técnico)</t>
-  </si>
-  <si>
     <t>ANÁLISIS GRANULOMÉTRICO POR TAMIZADO EN SUELOS</t>
   </si>
   <si>
@@ -197,6 +194,9 @@
   </si>
   <si>
     <t>NOTA:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT DESIGADA A:    </t>
   </si>
 </sst>
 </file>
@@ -205,9 +205,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;0&quot;0"/>
-    <numFmt numFmtId="167" formatCode="000\-&quot;26-LEM&quot;"/>
-    <numFmt numFmtId="168" formatCode="000\-&quot;26&quot;"/>
-    <numFmt numFmtId="169" formatCode="000&quot;-SU-26&quot;"/>
+    <numFmt numFmtId="165" formatCode="000\-&quot;26-LEM&quot;"/>
+    <numFmt numFmtId="166" formatCode="000\-&quot;26&quot;"/>
+    <numFmt numFmtId="167" formatCode="000&quot;-SU-26&quot;"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -500,7 +500,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -515,9 +515,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -537,7 +534,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -546,9 +543,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -559,38 +553,47 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -601,28 +604,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -631,22 +616,34 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -746,9 +743,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -786,9 +783,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -821,26 +818,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -873,26 +853,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1069,75 +1032,75 @@
   <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.109375" style="8" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="5.21875" style="8" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" style="21" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" style="8" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" style="8" customWidth="1"/>
-    <col min="8" max="9" width="13.88671875" style="8" customWidth="1"/>
-    <col min="10" max="10" width="18" style="8" customWidth="1"/>
-    <col min="11" max="12" width="11.44140625" style="8"/>
-    <col min="13" max="13" width="14.44140625" style="8" customWidth="1"/>
-    <col min="14" max="16384" width="11.44140625" style="8"/>
+    <col min="1" max="1" width="7.109375" style="7" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="5.21875" style="7" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" style="19" customWidth="1"/>
+    <col min="5" max="5" width="18.5546875" style="7" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="16.5546875" style="7" customWidth="1"/>
+    <col min="8" max="9" width="13.88671875" style="7" customWidth="1"/>
+    <col min="10" max="10" width="18" style="7" customWidth="1"/>
+    <col min="11" max="12" width="11.44140625" style="7"/>
+    <col min="13" max="13" width="14.44140625" style="7" customWidth="1"/>
+    <col min="14" max="16384" width="11.44140625" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23"/>
-      <c r="B1" s="24"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="49" t="s">
+      <c r="A1" s="41"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
       <c r="H1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
+      <c r="A2" s="44"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
       <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="26"/>
-      <c r="B3" s="27"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
       <c r="H3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="9">
         <v>46254</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29"/>
-      <c r="B4" s="30"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
+      <c r="A4" s="47"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
       <c r="H4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1146,65 +1109,65 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="10.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="12"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="11"/>
     </row>
     <row r="6" spans="1:10" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="38">
         <v>0</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="F6" s="13" t="s">
+      <c r="D6" s="38"/>
+      <c r="F6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="13">
         <v>0</v>
       </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
     </row>
     <row r="7" spans="1:10" ht="10.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="16"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="15"/>
     </row>
     <row r="8" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="45"/>
-      <c r="D8" s="46" t="s">
+      <c r="C8" s="40"/>
+      <c r="D8" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="47"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="48" t="s">
+      <c r="F8" s="50"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="43" t="s">
+      <c r="I8" s="22" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1212,39 +1175,39 @@
       <c r="A9" s="2">
         <v>1</v>
       </c>
-      <c r="B9" s="36">
+      <c r="B9" s="30">
         <v>3386</v>
       </c>
-      <c r="C9" s="37"/>
+      <c r="C9" s="31"/>
       <c r="D9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="39"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="41" t="s">
-        <v>35</v>
-      </c>
-      <c r="I9" s="42">
+      <c r="E9" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="28"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" s="21">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="36"/>
-      <c r="C10" s="37"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="31"/>
       <c r="D10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" s="39"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="41" t="s">
-        <v>36</v>
+        <v>20</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" s="28"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="20" t="s">
+        <v>35</v>
       </c>
       <c r="I10" s="2">
         <v>1</v>
@@ -1252,18 +1215,18 @@
     </row>
     <row r="11" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="36"/>
-      <c r="C11" s="37"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="31"/>
       <c r="D11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="39"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="41" t="s">
-        <v>37</v>
+        <v>21</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="28"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="20" t="s">
+        <v>36</v>
       </c>
       <c r="I11" s="2">
         <v>1</v>
@@ -1271,18 +1234,18 @@
     </row>
     <row r="12" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="37"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="31"/>
       <c r="D12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12" s="39"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="41" t="s">
-        <v>38</v>
+        <v>22</v>
+      </c>
+      <c r="E12" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="28"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="20" t="s">
+        <v>37</v>
       </c>
       <c r="I12" s="2">
         <v>1</v>
@@ -1290,18 +1253,18 @@
     </row>
     <row r="13" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="37"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="31"/>
       <c r="D13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="39"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="41" t="s">
-        <v>39</v>
+        <v>23</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="28"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="20" t="s">
+        <v>38</v>
       </c>
       <c r="I13" s="2">
         <v>1</v>
@@ -1309,18 +1272,18 @@
     </row>
     <row r="14" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="36"/>
-      <c r="C14" s="37"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="31"/>
       <c r="D14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="40"/>
-      <c r="H14" s="41" t="s">
-        <v>40</v>
+        <v>24</v>
+      </c>
+      <c r="E14" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="28"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="20" t="s">
+        <v>39</v>
       </c>
       <c r="I14" s="2">
         <v>1</v>
@@ -1328,33 +1291,33 @@
     </row>
     <row r="15" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="37"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="31"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="41"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="20"/>
       <c r="I15" s="2"/>
     </row>
     <row r="16" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>2</v>
       </c>
-      <c r="B16" s="36">
+      <c r="B16" s="30">
         <v>3386</v>
       </c>
-      <c r="C16" s="37"/>
+      <c r="C16" s="31"/>
       <c r="D16" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" s="39"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="41" t="s">
-        <v>41</v>
+        <v>25</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="28"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="20" t="s">
+        <v>40</v>
       </c>
       <c r="I16" s="2">
         <v>1</v>
@@ -1362,18 +1325,18 @@
     </row>
     <row r="17" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="36"/>
-      <c r="C17" s="37"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="31"/>
       <c r="D17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F17" s="39"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="41" t="s">
-        <v>42</v>
+        <v>26</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="28"/>
+      <c r="G17" s="29"/>
+      <c r="H17" s="20" t="s">
+        <v>41</v>
       </c>
       <c r="I17" s="2">
         <v>1</v>
@@ -1381,18 +1344,18 @@
     </row>
     <row r="18" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="36"/>
-      <c r="C18" s="37"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="31"/>
       <c r="D18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E18" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" s="39"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="41" t="s">
-        <v>43</v>
+        <v>27</v>
+      </c>
+      <c r="E18" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="28"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="20" t="s">
+        <v>42</v>
       </c>
       <c r="I18" s="2">
         <v>1</v>
@@ -1400,18 +1363,18 @@
     </row>
     <row r="19" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="36"/>
-      <c r="C19" s="37"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="31"/>
       <c r="D19" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F19" s="39"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="41" t="s">
-        <v>44</v>
+        <v>28</v>
+      </c>
+      <c r="E19" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="28"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="20" t="s">
+        <v>43</v>
       </c>
       <c r="I19" s="2">
         <v>1</v>
@@ -1419,18 +1382,18 @@
     </row>
     <row r="20" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="36"/>
-      <c r="C20" s="37"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="31"/>
       <c r="D20" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E20" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F20" s="39"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="41" t="s">
-        <v>45</v>
+        <v>29</v>
+      </c>
+      <c r="E20" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="28"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="20" t="s">
+        <v>44</v>
       </c>
       <c r="I20" s="2">
         <v>1</v>
@@ -1438,18 +1401,18 @@
     </row>
     <row r="21" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="36"/>
-      <c r="C21" s="37"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="31"/>
       <c r="D21" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E21" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" s="39"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="41" t="s">
-        <v>46</v>
+        <v>30</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="28"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="20" t="s">
+        <v>45</v>
       </c>
       <c r="I21" s="2">
         <v>1</v>
@@ -1457,18 +1420,18 @@
     </row>
     <row r="22" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="36"/>
-      <c r="C22" s="37"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="31"/>
       <c r="D22" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E22" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F22" s="39"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="41" t="s">
-        <v>47</v>
+        <v>31</v>
+      </c>
+      <c r="E22" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="28"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="20" t="s">
+        <v>46</v>
       </c>
       <c r="I22" s="2">
         <v>1</v>
@@ -1476,18 +1439,18 @@
     </row>
     <row r="23" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="36"/>
-      <c r="C23" s="37"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="31"/>
       <c r="D23" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F23" s="39"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="41" t="s">
-        <v>48</v>
+        <v>32</v>
+      </c>
+      <c r="E23" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" s="28"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="20" t="s">
+        <v>47</v>
       </c>
       <c r="I23" s="2">
         <v>1</v>
@@ -1495,18 +1458,18 @@
     </row>
     <row r="24" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="31"/>
       <c r="D24" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E24" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="39"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="41" t="s">
-        <v>49</v>
+        <v>33</v>
+      </c>
+      <c r="E24" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="28"/>
+      <c r="G24" s="29"/>
+      <c r="H24" s="20" t="s">
+        <v>48</v>
       </c>
       <c r="I24" s="2">
         <v>1</v>
@@ -1514,80 +1477,80 @@
     </row>
     <row r="25" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="36"/>
-      <c r="C25" s="37"/>
+      <c r="B25" s="30"/>
+      <c r="C25" s="31"/>
       <c r="D25" s="2"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="41"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="28"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="20"/>
       <c r="I25" s="2"/>
     </row>
     <row r="26" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="36"/>
-      <c r="C26" s="37"/>
+      <c r="B26" s="30"/>
+      <c r="C26" s="31"/>
       <c r="D26" s="2"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="41"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="20"/>
       <c r="I26" s="2"/>
     </row>
     <row r="27" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="36"/>
-      <c r="C27" s="37"/>
+      <c r="B27" s="30"/>
+      <c r="C27" s="31"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="41"/>
+      <c r="E27" s="27"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="20"/>
       <c r="I27" s="2"/>
     </row>
     <row r="28" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="36"/>
-      <c r="C28" s="37"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="31"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="41"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="20"/>
       <c r="I28" s="2"/>
     </row>
     <row r="29" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="36"/>
-      <c r="C29" s="37"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="31"/>
       <c r="D29" s="2"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="40"/>
-      <c r="H29" s="41"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="20"/>
       <c r="I29" s="2"/>
     </row>
     <row r="30" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="36"/>
-      <c r="C30" s="37"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="31"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="41"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="29"/>
+      <c r="H30" s="20"/>
       <c r="I30" s="2"/>
     </row>
     <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D31" s="8"/>
+      <c r="D31" s="7"/>
     </row>
     <row r="32" spans="1:9" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="33" t="s">
+      <c r="A32" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="34"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="35"/>
+      <c r="B32" s="35"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="5">
         <v>46251</v>
       </c>
@@ -1605,55 +1568,101 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="51" t="s">
+      <c r="A33" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="35"/>
+      <c r="C33" s="35"/>
+      <c r="D33" s="35"/>
+      <c r="E33" s="35"/>
+      <c r="F33" s="35"/>
+      <c r="G33" s="35"/>
+      <c r="H33" s="35"/>
+      <c r="I33" s="35"/>
+    </row>
+    <row r="34" spans="1:9" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="26"/>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="26"/>
+    </row>
+    <row r="35" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D35" s="7"/>
+    </row>
+    <row r="36" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="E36" s="33"/>
+      <c r="F36" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="34"/>
-      <c r="H33" s="34"/>
-      <c r="I33" s="34"/>
-    </row>
-    <row r="34" spans="1:9" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="50"/>
-      <c r="B34" s="50"/>
-      <c r="C34" s="50"/>
-      <c r="D34" s="50"/>
-      <c r="E34" s="50"/>
-      <c r="F34" s="50"/>
-      <c r="G34" s="50"/>
-      <c r="H34" s="50"/>
-      <c r="I34" s="50"/>
-    </row>
-    <row r="35" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D35" s="8"/>
-    </row>
-    <row r="36" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B36" s="7"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="E36" s="17"/>
-      <c r="F36" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="32"/>
     </row>
     <row r="43" spans="1:9" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="44" spans="1:9" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G44" s="18"/>
+      <c r="G44" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="56">
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="D1:G4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:C4"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
     <mergeCell ref="A34:I34"/>
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="B30:C30"/>
@@ -1663,53 +1672,7 @@
     <mergeCell ref="E26:G26"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="E27:G27"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A32:D32"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="D1:G4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:C4"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="E9:G9"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
fix(templates): sincronizar nueva version de plantilla OT Suelo y Agregado
</commit_message>
<xml_diff>
--- a/app/templates/OT/OT-SU-Y-AG/OT-0000-Geofal.xlsx
+++ b/app/templates/OT/OT-SU-Y-AG/OT-0000-Geofal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\OT\OT-SU-Y-AG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28D30F3E-C883-4009-89AB-A80F22AE44C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49E29017-F877-4039-A481-83F46DF974D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7CAA3784-AC6A-4491-9DAE-0EC89CC1DDD5}"/>
+    <workbookView xWindow="0" yWindow="1536" windowWidth="23040" windowHeight="10920" xr2:uid="{7CAA3784-AC6A-4491-9DAE-0EC89CC1DDD5}"/>
   </bookViews>
   <sheets>
     <sheet name="HOJA 1 (2)" sheetId="3" r:id="rId1"/>
@@ -571,8 +571,11 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -583,11 +586,47 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -604,46 +643,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1047,15 +1047,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="41"/>
-      <c r="B1" s="42"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="37" t="s">
+      <c r="A1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
       <c r="H1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1064,13 +1064,13 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="44"/>
-      <c r="B2" s="45"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
+      <c r="A2" s="38"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
       <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1079,28 +1079,28 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="44"/>
-      <c r="B3" s="45"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
+      <c r="A3" s="38"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
       <c r="H3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I3" s="9">
-        <v>46254</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="47"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
+      <c r="A4" s="41"/>
+      <c r="B4" s="42"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
       <c r="H4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1124,10 +1124,10 @@
       <c r="B6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="32">
         <v>0</v>
       </c>
-      <c r="D6" s="38"/>
+      <c r="D6" s="32"/>
       <c r="F6" s="12" t="s">
         <v>7</v>
       </c>
@@ -1152,18 +1152,18 @@
       <c r="A8" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="40"/>
+      <c r="C8" s="34"/>
       <c r="D8" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="39" t="s">
+      <c r="E8" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="50"/>
-      <c r="G8" s="40"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="34"/>
       <c r="H8" s="24" t="s">
         <v>16</v>
       </c>
@@ -1175,18 +1175,18 @@
       <c r="A9" s="2">
         <v>1</v>
       </c>
-      <c r="B9" s="30">
+      <c r="B9" s="26">
         <v>3386</v>
       </c>
-      <c r="C9" s="31"/>
+      <c r="C9" s="27"/>
       <c r="D9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="28"/>
-      <c r="G9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="30"/>
       <c r="H9" s="20" t="s">
         <v>34</v>
       </c>
@@ -1196,16 +1196,16 @@
     </row>
     <row r="10" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="31"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="27"/>
       <c r="D10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E10" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="28"/>
-      <c r="G10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="30"/>
       <c r="H10" s="20" t="s">
         <v>35</v>
       </c>
@@ -1215,16 +1215,16 @@
     </row>
     <row r="11" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="30"/>
-      <c r="C11" s="31"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="27"/>
       <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="E11" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="28"/>
-      <c r="G11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="30"/>
       <c r="H11" s="20" t="s">
         <v>36</v>
       </c>
@@ -1234,16 +1234,16 @@
     </row>
     <row r="12" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="30"/>
-      <c r="C12" s="31"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="27"/>
       <c r="D12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="27" t="s">
+      <c r="E12" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="28"/>
-      <c r="G12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="30"/>
       <c r="H12" s="20" t="s">
         <v>37</v>
       </c>
@@ -1253,16 +1253,16 @@
     </row>
     <row r="13" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="30"/>
-      <c r="C13" s="31"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="27"/>
       <c r="D13" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="28"/>
-      <c r="G13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="30"/>
       <c r="H13" s="20" t="s">
         <v>38</v>
       </c>
@@ -1272,16 +1272,16 @@
     </row>
     <row r="14" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="31"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="27"/>
       <c r="D14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="28"/>
-      <c r="G14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="30"/>
       <c r="H14" s="20" t="s">
         <v>39</v>
       </c>
@@ -1291,12 +1291,12 @@
     </row>
     <row r="15" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="31"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="27"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="29"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="30"/>
       <c r="H15" s="20"/>
       <c r="I15" s="2"/>
     </row>
@@ -1304,18 +1304,18 @@
       <c r="A16" s="2">
         <v>2</v>
       </c>
-      <c r="B16" s="30">
+      <c r="B16" s="26">
         <v>3386</v>
       </c>
-      <c r="C16" s="31"/>
+      <c r="C16" s="27"/>
       <c r="D16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="28"/>
-      <c r="G16" s="29"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="30"/>
       <c r="H16" s="20" t="s">
         <v>40</v>
       </c>
@@ -1325,16 +1325,16 @@
     </row>
     <row r="17" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="31"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="27"/>
       <c r="D17" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E17" s="27" t="s">
+      <c r="E17" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F17" s="28"/>
-      <c r="G17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="30"/>
       <c r="H17" s="20" t="s">
         <v>41</v>
       </c>
@@ -1344,16 +1344,16 @@
     </row>
     <row r="18" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="27"/>
       <c r="D18" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="27" t="s">
+      <c r="E18" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="28"/>
-      <c r="G18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="30"/>
       <c r="H18" s="20" t="s">
         <v>42</v>
       </c>
@@ -1363,16 +1363,16 @@
     </row>
     <row r="19" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="31"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="27"/>
       <c r="D19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F19" s="28"/>
-      <c r="G19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="30"/>
       <c r="H19" s="20" t="s">
         <v>43</v>
       </c>
@@ -1382,16 +1382,16 @@
     </row>
     <row r="20" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="31"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="27"/>
       <c r="D20" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="27" t="s">
+      <c r="E20" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="28"/>
-      <c r="G20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="30"/>
       <c r="H20" s="20" t="s">
         <v>44</v>
       </c>
@@ -1401,16 +1401,16 @@
     </row>
     <row r="21" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="30"/>
-      <c r="C21" s="31"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="27"/>
       <c r="D21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="27" t="s">
+      <c r="E21" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="28"/>
-      <c r="G21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="30"/>
       <c r="H21" s="20" t="s">
         <v>45</v>
       </c>
@@ -1420,16 +1420,16 @@
     </row>
     <row r="22" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="31"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="27"/>
       <c r="D22" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="27" t="s">
+      <c r="E22" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F22" s="28"/>
-      <c r="G22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="30"/>
       <c r="H22" s="20" t="s">
         <v>46</v>
       </c>
@@ -1439,16 +1439,16 @@
     </row>
     <row r="23" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="31"/>
+      <c r="B23" s="26"/>
+      <c r="C23" s="27"/>
       <c r="D23" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="27" t="s">
+      <c r="E23" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F23" s="28"/>
-      <c r="G23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="30"/>
       <c r="H23" s="20" t="s">
         <v>47</v>
       </c>
@@ -1458,16 +1458,16 @@
     </row>
     <row r="24" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="31"/>
+      <c r="B24" s="26"/>
+      <c r="C24" s="27"/>
       <c r="D24" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="27" t="s">
+      <c r="E24" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="28"/>
-      <c r="G24" s="29"/>
+      <c r="F24" s="29"/>
+      <c r="G24" s="30"/>
       <c r="H24" s="20" t="s">
         <v>48</v>
       </c>
@@ -1477,67 +1477,67 @@
     </row>
     <row r="25" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="30"/>
-      <c r="C25" s="31"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="27"/>
       <c r="D25" s="2"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="29"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="30"/>
       <c r="H25" s="20"/>
       <c r="I25" s="2"/>
     </row>
     <row r="26" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="30"/>
-      <c r="C26" s="31"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="27"/>
       <c r="D26" s="2"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="29"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="30"/>
       <c r="H26" s="20"/>
       <c r="I26" s="2"/>
     </row>
     <row r="27" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="30"/>
-      <c r="C27" s="31"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="27"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="29"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="30"/>
       <c r="H27" s="20"/>
       <c r="I27" s="2"/>
     </row>
     <row r="28" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="30"/>
-      <c r="C28" s="31"/>
+      <c r="B28" s="26"/>
+      <c r="C28" s="27"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="29"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="30"/>
       <c r="H28" s="20"/>
       <c r="I28" s="2"/>
     </row>
     <row r="29" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="30"/>
-      <c r="C29" s="31"/>
+      <c r="B29" s="26"/>
+      <c r="C29" s="27"/>
       <c r="D29" s="2"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="29"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="30"/>
       <c r="H29" s="20"/>
       <c r="I29" s="2"/>
     </row>
     <row r="30" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="30"/>
-      <c r="C30" s="31"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="27"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="29"/>
+      <c r="E30" s="28"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="30"/>
       <c r="H30" s="20"/>
       <c r="I30" s="2"/>
     </row>
@@ -1545,12 +1545,12 @@
       <c r="D31" s="7"/>
     </row>
     <row r="32" spans="1:9" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="34" t="s">
+      <c r="A32" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="35"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="36"/>
+      <c r="B32" s="48"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="49"/>
       <c r="E32" s="5">
         <v>46251</v>
       </c>
@@ -1571,45 +1571,45 @@
       <c r="A33" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
+      <c r="B33" s="48"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="48"/>
+      <c r="G33" s="48"/>
+      <c r="H33" s="48"/>
+      <c r="I33" s="48"/>
     </row>
     <row r="34" spans="1:9" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="26"/>
-      <c r="B34" s="26"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="26"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
+      <c r="A34" s="50"/>
+      <c r="B34" s="50"/>
+      <c r="C34" s="50"/>
+      <c r="D34" s="50"/>
+      <c r="E34" s="50"/>
+      <c r="F34" s="50"/>
+      <c r="G34" s="50"/>
+      <c r="H34" s="50"/>
+      <c r="I34" s="50"/>
     </row>
     <row r="35" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D35" s="7"/>
     </row>
     <row r="36" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="32" t="s">
+      <c r="A36" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="33" t="s">
+      <c r="B36" s="45"/>
+      <c r="C36" s="45"/>
+      <c r="D36" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="E36" s="33"/>
-      <c r="F36" s="32" t="s">
+      <c r="E36" s="46"/>
+      <c r="F36" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="32"/>
+      <c r="G36" s="45"/>
+      <c r="H36" s="45"/>
+      <c r="I36" s="45"/>
     </row>
     <row r="43" spans="1:9" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="44" spans="1:9" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
@@ -1617,13 +1617,42 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="D1:G4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:C4"/>
-    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="E14:G14"/>
     <mergeCell ref="F36:G36"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="D36:E36"/>
@@ -1633,46 +1662,17 @@
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="B33:I33"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="E14:G14"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
     <mergeCell ref="A34:I34"/>
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="E30:G30"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="D1:G4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:C4"/>
+    <mergeCell ref="E8:G8"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>